<commit_message>
Add target testing toggle, fix SAP level RIA calculation, AICPA MUS formula
</commit_message>
<xml_diff>
--- a/outputs/Revenue_Test_Workpaper.xlsx
+++ b/outputs/Revenue_Test_Workpaper.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Population Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Target Testing'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Target Testing'!$A$2:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MUS Sample'!$A$2:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Population Summary'!$A$1:$E$1</definedName>
   </definedNames>
@@ -90,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,11 +102,17 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -116,9 +122,6 @@
     </xf>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -493,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -526,146 +529,210 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>500000</v>
+        <v>2000000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Inherent Risk</t>
+          <t>Target Testing</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Lower</t>
+          <t>Disabled</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Control Risk</t>
+          <t>Target Testing Note</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Higher</t>
+          <t>Target testing not performed - MUS applied to full population</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>SAP Level</t>
+          <t>Inherent Risk</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Persuasive</t>
+          <t>Lower</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Confidence Level</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>90</v>
+          <t>Control Risk</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Higher</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Cutoff Date</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>45473</v>
+          <t>SAP Level</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Persuasive</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Test Negatives</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="b">
-        <v>0</v>
+          <t>Confidence Level</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Run ID</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>08e477fb-aa07-4873-ad28-ccae50a8d580</t>
-        </is>
+          <t>RIA (Risk of Incorrect Acceptance)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Date/Time of run</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>46135.94092807861</v>
+          <t>Confidence Factor (Poisson, 0 expected misstatements)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Total population count</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>50</v>
+          <t>MUS Sample Size Formula</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>CEILING((Population Value × Confidence Factor) / Tolerable Misstatement)</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Total population value</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>21218088.66</v>
+          <t>MUS Sample Size</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Less Target Tested Value</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>17949446.31</v>
+          <t>Cutoff Date</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>45473</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Residual Population Value used for MUS</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>3268642.35</v>
+          <t>Test Negatives</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Run ID</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>24856f95-4fa1-4ad5-bce2-210aff67637c</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Date/Time of run</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>46139.86147495517</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Total population count</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Total population value</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>21218088.66</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Less Target Tested Value</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Residual Population Value used for MUS (positive amounts)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>21218088.66</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
           <t>Target testing threshold</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
-        <v>250000</v>
-      </c>
+      <c r="B23" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -678,733 +745,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Target testing not performed - MUS applied to full population</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Invoice Number</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Threshold Used</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Reason Selected</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00043</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="n">
-        <v>45433</v>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Northwind Distribution LLC</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>340461.42</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00044</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>45321</v>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Orchard Financial Services</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>442509.44</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-LARGE-004</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>45421</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Contoso Retail Group</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>2523407.5</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-LARGE-002</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>45292</v>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Pioneer Telecom</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>2532742.65</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00019</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>45309</v>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Northwind Distribution LLC</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>330970.4</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00007</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>45435</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>BlueRock Logistics Inc.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>358293.79</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00023</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>45382</v>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>BlueRock Logistics Inc.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>335417.41</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-LARGE-005</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>45368</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Orchard Financial Services</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>1888410.04</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-LARGE-001</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>45367</v>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Summit IT Services</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>1276776.07</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00014</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>45446</v>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Redwood Healthcare Partners</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>403757.01</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00017</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>45452</v>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Evergreen Construction Ltd.</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>442840.42</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00031</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>45346</v>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Evergreen Construction Ltd.</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>438307.45</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00029</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>45306</v>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>BlueRock Logistics Inc.</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>411079.49</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00003</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>45318</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Orchard Financial Services</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>370593.2</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00027</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>45361</v>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Orchard Financial Services</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>344392.82</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00006</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>45351</v>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Crescent Energy Solutions</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>301407.35</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00036</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>45441</v>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Summit IT Services</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>449013.62</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00004</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>45431</v>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Contoso Retail Group</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>295655.76</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00016</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>45388</v>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Contoso Retail Group</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>276468.28</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00020</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>45366</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Contoso Retail Group</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>427803.54</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-LARGE-003</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="n">
-        <v>45359</v>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Crescent Energy Solutions</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>2333433.85</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00032</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>45372</v>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>BlueRock Logistics Inc.</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>328063.89</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00024</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>45471</v>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Orchard Financial Services</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>324369.66</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00010</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>45293</v>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Fabrikam Manufacturing Co.</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>349371.56</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>INV-2024-00013</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>45316</v>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Apex Industrial Supply</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>423899.69</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Amount exceeds threshold</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="3" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Total value</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="n">
-        <v>17949446.31</v>
-      </c>
-      <c r="F28" s="3" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A2:F2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1415,23 +810,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>MUS sample drawn from residual population (total less target-tested items).</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>MUS sample drawn from full population (target testing not performed).</t>
         </is>
       </c>
     </row>
@@ -1483,23 +878,23 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>INV-2024-00028</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>45348</v>
+          <t>INV-2024-LARGE-004</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>45421</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Orchard Financial Services</t>
+          <t>Contoso Retail Group</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>162817.08</v>
+        <v>2523407.5</v>
       </c>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n">
-        <v>466948.9071428571</v>
+        <v>1928917.150909091</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
@@ -1513,23 +908,23 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>INV-2024-00009</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>45406</v>
+          <t>INV-2024-LARGE-002</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>45292</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Evergreen Construction Ltd.</t>
+          <t>Pioneer Telecom</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>139817.16</v>
+        <v>2532742.65</v>
       </c>
       <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="n">
-        <v>466948.9071428571</v>
+        <v>1928917.150909091</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
@@ -1543,23 +938,23 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>INV-2024-00030</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>45372</v>
+          <t>INV-2024-00023</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>45382</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Summit IT Services</t>
+          <t>BlueRock Logistics Inc.</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>134602.7</v>
+        <v>335417.41</v>
       </c>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n">
-        <v>466948.9071428571</v>
+        <v>1928917.150909091</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -1573,11 +968,11 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>INV-2024-00045</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>45360</v>
+          <t>INV-2024-LARGE-005</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>45368</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
@@ -1585,11 +980,11 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>170747.56</v>
+        <v>1888410.04</v>
       </c>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n">
-        <v>466948.9071428571</v>
+        <v>1928917.150909091</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -1603,23 +998,23 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>INV-2024-00033</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>45393</v>
+          <t>INV-2024-00014</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>45446</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Orchard Financial Services</t>
+          <t>Redwood Healthcare Partners</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>229967.07</v>
+        <v>403757.01</v>
       </c>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n">
-        <v>466948.9071428571</v>
+        <v>1928917.150909091</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
@@ -1633,11 +1028,11 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>INV-2024-00002</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>45362</v>
+          <t>INV-2024-00029</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>45306</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
@@ -1645,11 +1040,11 @@
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>112382.16</v>
+        <v>411079.49</v>
       </c>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n">
-        <v>466948.9071428571</v>
+        <v>1928917.150909091</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -1663,11 +1058,11 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>INV-2024-00035</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>45435</v>
+          <t>INV-2024-00006</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>45351</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
@@ -1675,11 +1070,11 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>132108.06</v>
+        <v>301407.35</v>
       </c>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n">
-        <v>466948.9071428571</v>
+        <v>1928917.150909091</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
@@ -1688,40 +1083,100 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="4" t="n"/>
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>INV-2024-LARGE-003</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>45359</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Crescent Energy Solutions</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>2333433.85</v>
+      </c>
       <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="3" t="n"/>
+      <c r="G10" s="4" t="n">
+        <v>1928917.150909091</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Residual population MUS: cumulative value crossed sampling interval point</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>INV-2024-00010</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>45293</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Fabrikam Manufacturing Co.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>349371.56</v>
+      </c>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n">
+        <v>1928917.150909091</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Residual population MUS: cumulative value crossed sampling interval point</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Sample size</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="C13" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Total value</t>
         </is>
       </c>
-      <c r="E11" s="9" t="n">
-        <v>1082441.79</v>
-      </c>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="3" t="n"/>
+      <c r="E13" s="11" t="n">
+        <v>11079026.86</v>
+      </c>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:H2"/>
@@ -1750,13 +1205,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Pre-cutoff transactions (before 30/06/2024)</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="D1" s="12" t="n"/>
+      <c r="B1" s="12" t="n"/>
+      <c r="D1" s="13" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1764,7 +1219,7 @@
           <t>Invoice Number</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -1774,7 +1229,7 @@
           <t>Customer</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -1796,7 +1251,7 @@
           <t>INV-2024-00024</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n">
+      <c r="B3" s="12" t="n">
         <v>45471</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1804,7 +1259,7 @@
           <t>Orchard Financial Services</t>
         </is>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="13" t="n">
         <v>324369.66</v>
       </c>
       <c r="E3" t="inlineStr">
@@ -1819,7 +1274,7 @@
           <t>INV-2024-00008</t>
         </is>
       </c>
-      <c r="B4" s="11" t="n">
+      <c r="B4" s="12" t="n">
         <v>45471</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1827,7 +1282,7 @@
           <t>Crescent Energy Solutions</t>
         </is>
       </c>
-      <c r="D4" s="12" t="n">
+      <c r="D4" s="13" t="n">
         <v>210340.39</v>
       </c>
       <c r="E4" t="inlineStr">
@@ -1842,7 +1297,7 @@
           <t>INV-2024-00001</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="12" t="n">
         <v>45455</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1850,7 +1305,7 @@
           <t>Contoso Retail Group</t>
         </is>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="13" t="n">
         <v>13480.37</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -1865,7 +1320,7 @@
           <t>INV-2024-00022</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="12" t="n">
         <v>45454</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -1873,7 +1328,7 @@
           <t>Apex Industrial Supply</t>
         </is>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="13" t="n">
         <v>82164.39</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -1888,7 +1343,7 @@
           <t>INV-2024-00017</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="12" t="n">
         <v>45452</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1896,7 +1351,7 @@
           <t>Evergreen Construction Ltd.</t>
         </is>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="13" t="n">
         <v>442840.42</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -1906,17 +1361,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="11" t="n"/>
-      <c r="D8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="D8" s="13" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Post-cutoff transactions (after 30/06/2024)</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="D9" s="12" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="D9" s="13" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1924,7 +1379,7 @@
           <t>Invoice Number</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -1934,7 +1389,7 @@
           <t>Customer</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -1972,7 +1427,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="29" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2008,7 +1463,7 @@
           <t>INV-2024-00040</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="6" t="n">
         <v>45332</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -2031,7 +1486,7 @@
           <t>INV-2024-00028</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="6" t="n">
         <v>45348</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -2044,7 +1499,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>MUS</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2054,7 +1509,7 @@
           <t>INV-2024-00043</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="6" t="n">
         <v>45433</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -2067,7 +1522,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2077,7 +1532,7 @@
           <t>INV-2024-00044</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>45321</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -2090,7 +1545,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2100,7 +1555,7 @@
           <t>INV-2024-00042</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>45411</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -2123,7 +1578,7 @@
           <t>INV-2024-LARGE-004</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <v>45421</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -2136,7 +1591,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -2146,7 +1601,7 @@
           <t>INV-2024-LARGE-002</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <v>45292</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -2159,7 +1614,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -2169,7 +1624,7 @@
           <t>INV-2024-00019</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>45309</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -2182,7 +1637,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2192,7 +1647,7 @@
           <t>INV-2024-00007</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>45435</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -2205,7 +1660,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2215,7 +1670,7 @@
           <t>INV-2024-00023</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="6" t="n">
         <v>45382</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -2228,7 +1683,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -2238,7 +1693,7 @@
           <t>INV-2024-00015</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="6" t="n">
         <v>45409</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -2261,7 +1716,7 @@
           <t>INV-2024-00012</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="6" t="n">
         <v>45378</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -2284,7 +1739,7 @@
           <t>INV-2024-LARGE-005</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="6" t="n">
         <v>45368</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -2297,7 +1752,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -2307,7 +1762,7 @@
           <t>INV-2024-00037</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="6" t="n">
         <v>45394</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -2330,7 +1785,7 @@
           <t>INV-2024-LARGE-001</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="6" t="n">
         <v>45367</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -2343,7 +1798,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2353,7 +1808,7 @@
           <t>INV-2024-00014</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="6" t="n">
         <v>45446</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -2366,7 +1821,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -2376,7 +1831,7 @@
           <t>INV-2024-00017</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B18" s="6" t="n">
         <v>45452</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -2389,7 +1844,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Target/Cutoff</t>
+          <t>Cutoff</t>
         </is>
       </c>
     </row>
@@ -2399,7 +1854,7 @@
           <t>INV-2024-00009</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B19" s="6" t="n">
         <v>45406</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -2412,7 +1867,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>MUS</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2422,7 +1877,7 @@
           <t>INV-2024-00041</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B20" s="6" t="n">
         <v>45308</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -2445,7 +1900,7 @@
           <t>INV-2024-00026</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B21" s="6" t="n">
         <v>45354</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -2468,7 +1923,7 @@
           <t>INV-2024-00030</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
+      <c r="B22" s="6" t="n">
         <v>45372</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -2481,7 +1936,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>MUS</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2491,7 +1946,7 @@
           <t>INV-2024-00022</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
+      <c r="B23" s="6" t="n">
         <v>45454</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -2514,7 +1969,7 @@
           <t>INV-2024-00031</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B24" s="6" t="n">
         <v>45346</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -2527,7 +1982,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2537,7 +1992,7 @@
           <t>INV-2024-00005</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B25" s="6" t="n">
         <v>45300</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -2560,7 +2015,7 @@
           <t>INV-2024-00029</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
+      <c r="B26" s="6" t="n">
         <v>45306</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -2573,7 +2028,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2038,7 @@
           <t>INV-2024-00018</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
+      <c r="B27" s="6" t="n">
         <v>45384</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -2606,7 +2061,7 @@
           <t>INV-2024-00025</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
+      <c r="B28" s="6" t="n">
         <v>45447</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -2629,7 +2084,7 @@
           <t>INV-2024-00003</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
+      <c r="B29" s="6" t="n">
         <v>45318</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -2642,7 +2097,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2107,7 @@
           <t>INV-2024-00027</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n">
+      <c r="B30" s="6" t="n">
         <v>45361</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -2665,7 +2120,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2130,7 @@
           <t>INV-2024-00045</t>
         </is>
       </c>
-      <c r="B31" s="5" t="n">
+      <c r="B31" s="6" t="n">
         <v>45360</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2688,7 +2143,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>MUS</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2153,7 @@
           <t>INV-2024-00038</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
+      <c r="B32" s="6" t="n">
         <v>45327</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2721,7 +2176,7 @@
           <t>INV-2024-00033</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n">
+      <c r="B33" s="6" t="n">
         <v>45393</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2734,7 +2189,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>MUS</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2199,7 @@
           <t>INV-2024-00006</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n">
+      <c r="B34" s="6" t="n">
         <v>45351</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2757,7 +2212,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2222,7 @@
           <t>INV-2024-00036</t>
         </is>
       </c>
-      <c r="B35" s="5" t="n">
+      <c r="B35" s="6" t="n">
         <v>45441</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2780,7 +2235,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2790,7 +2245,7 @@
           <t>INV-2024-00004</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
+      <c r="B36" s="6" t="n">
         <v>45431</v>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2803,7 +2258,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2268,7 @@
           <t>INV-2024-00016</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
+      <c r="B37" s="6" t="n">
         <v>45388</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2826,7 +2281,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2291,7 @@
           <t>INV-2024-00020</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n">
+      <c r="B38" s="6" t="n">
         <v>45366</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2849,7 +2304,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2314,7 @@
           <t>INV-2024-LARGE-003</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n">
+      <c r="B39" s="6" t="n">
         <v>45359</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2872,7 +2327,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2337,7 @@
           <t>INV-2024-00008</t>
         </is>
       </c>
-      <c r="B40" s="5" t="n">
+      <c r="B40" s="6" t="n">
         <v>45471</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2905,7 +2360,7 @@
           <t>INV-2024-00002</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n">
+      <c r="B41" s="6" t="n">
         <v>45362</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2918,7 +2373,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>MUS</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2383,7 @@
           <t>INV-2024-00032</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n">
+      <c r="B42" s="6" t="n">
         <v>45372</v>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2941,7 +2396,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2406,7 @@
           <t>INV-2024-00021</t>
         </is>
       </c>
-      <c r="B43" s="5" t="n">
+      <c r="B43" s="6" t="n">
         <v>45317</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2974,7 +2429,7 @@
           <t>INV-2024-00039</t>
         </is>
       </c>
-      <c r="B44" s="5" t="n">
+      <c r="B44" s="6" t="n">
         <v>45304</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2997,7 +2452,7 @@
           <t>INV-2024-00001</t>
         </is>
       </c>
-      <c r="B45" s="5" t="n">
+      <c r="B45" s="6" t="n">
         <v>45455</v>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -3020,7 +2475,7 @@
           <t>INV-2024-00034</t>
         </is>
       </c>
-      <c r="B46" s="5" t="n">
+      <c r="B46" s="6" t="n">
         <v>45359</v>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -3043,7 +2498,7 @@
           <t>INV-2024-00035</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n">
+      <c r="B47" s="6" t="n">
         <v>45435</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -3056,7 +2511,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>MUS</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>
@@ -3066,7 +2521,7 @@
           <t>INV-2024-00011</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n">
+      <c r="B48" s="6" t="n">
         <v>45379</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -3089,7 +2544,7 @@
           <t>INV-2024-00024</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
+      <c r="B49" s="6" t="n">
         <v>45471</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -3102,7 +2557,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Target/Cutoff</t>
+          <t>Cutoff</t>
         </is>
       </c>
     </row>
@@ -3112,7 +2567,7 @@
           <t>INV-2024-00010</t>
         </is>
       </c>
-      <c r="B50" s="5" t="n">
+      <c r="B50" s="6" t="n">
         <v>45293</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3125,7 +2580,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>MUS</t>
         </is>
       </c>
     </row>
@@ -3135,7 +2590,7 @@
           <t>INV-2024-00013</t>
         </is>
       </c>
-      <c r="B51" s="5" t="n">
+      <c r="B51" s="6" t="n">
         <v>45316</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3148,7 +2603,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Not Selected</t>
         </is>
       </c>
     </row>

</xml_diff>